<commit_message>
Update du mapping EvenementCDAFHIR e2862df637d104280a6743209426dfcfb9262290
</commit_message>
<xml_diff>
--- a/htr-mapping-CDA/FHIR/ig/mappingEvenementCDAFHIR.xlsx
+++ b/htr-mapping-CDA/FHIR/ig/mappingEvenementCDAFHIR.xlsx
@@ -58,7 +58,7 @@
     <t>Date</t>
   </si>
   <si>
-    <t>2025-04-28T09:28:28+00:00</t>
+    <t>2025-05-14T12:14:19+00:00</t>
   </si>
   <si>
     <t>Publisher</t>
@@ -177,13 +177,13 @@
     <t>Composition.event.period</t>
   </si>
   <si>
-    <t>Composition.event.detail</t>
-  </si>
-  <si>
-    <t>Composition.event.detail.PractitionerRole.code</t>
-  </si>
-  <si>
-    <t>Composition.event.detail.PractitionerRole.Practitioner</t>
+    <t>Composition.event.extension:perfomer.PractitionerRole</t>
+  </si>
+  <si>
+    <t>Composition.event.extension:perfomer.PractitionerRole.code</t>
+  </si>
+  <si>
+    <t>Composition.event.extension:perfomer.PractitionerRole.Practitioner</t>
   </si>
 </sst>
 </file>

</xml_diff>